<commit_message>
Updated plasma source database
</commit_message>
<xml_diff>
--- a/plasma_sources.xlsx
+++ b/plasma_sources.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\V.Ravavarapu\PycharmProjects\PythonProject_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A5B344-9D68-4C3D-9599-2F2A5489E6A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF19ACED-55E4-48BE-AF64-5B00960A4230}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Source_ID</t>
   </si>
@@ -34,40 +34,52 @@
     <t>Current_Density_mAcm2</t>
   </si>
   <si>
-    <t>LS02</t>
-  </si>
-  <si>
-    <t>DN01</t>
-  </si>
-  <si>
-    <t>DN</t>
-  </si>
-  <si>
-    <t>IS01</t>
-  </si>
-  <si>
-    <t>IS</t>
-  </si>
-  <si>
-    <t>RS01</t>
-  </si>
-  <si>
-    <t>RS</t>
-  </si>
-  <si>
-    <t>LS 1600x200</t>
-  </si>
-  <si>
-    <t>LS 1800x200</t>
-  </si>
-  <si>
     <t>Power_kW</t>
   </si>
   <si>
-    <t>Version</t>
-  </si>
-  <si>
     <t>coil current (mA)</t>
+  </si>
+  <si>
+    <t>Source_type</t>
+  </si>
+  <si>
+    <t>COPRA DN</t>
+  </si>
+  <si>
+    <t>COPRA IS</t>
+  </si>
+  <si>
+    <t>COPRA RS</t>
+  </si>
+  <si>
+    <t>COPRA LS</t>
+  </si>
+  <si>
+    <t>DN200</t>
+  </si>
+  <si>
+    <t>IS200</t>
+  </si>
+  <si>
+    <t>DN300</t>
+  </si>
+  <si>
+    <t>DN400</t>
+  </si>
+  <si>
+    <t>IS250</t>
+  </si>
+  <si>
+    <t>RS300</t>
+  </si>
+  <si>
+    <t>LS1600x200</t>
+  </si>
+  <si>
+    <t>LS1800x200</t>
+  </si>
+  <si>
+    <t>version</t>
   </si>
 </sst>
 </file>
@@ -551,7 +563,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -559,7 +571,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -915,207 +932,243 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="20.21875" customWidth="1"/>
     <col min="4" max="4" width="27" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="17.88671875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="17.21875" customWidth="1"/>
+    <col min="6" max="6" width="24" style="4" customWidth="1"/>
+    <col min="7" max="7" width="15.21875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="16" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>15</v>
+      <c r="G1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>581</v>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="1">
+        <v>254</v>
+      </c>
+      <c r="D2" s="1">
+        <v>581</v>
+      </c>
+      <c r="E2" s="2">
         <v>33</v>
       </c>
-      <c r="D2" s="1">
+      <c r="F2" s="2">
         <v>0.98</v>
       </c>
-      <c r="E2" s="1">
+      <c r="G2" s="3">
         <v>10</v>
       </c>
-      <c r="F2" s="2">
-        <v>341</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="H2" s="3">
         <v>1500</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1">
+        <v>265</v>
+      </c>
+      <c r="D3" s="1">
         <v>567</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="E3" s="2">
         <v>28</v>
       </c>
-      <c r="D3" s="1">
+      <c r="F3" s="2">
         <v>1.25</v>
       </c>
-      <c r="E3" s="1">
+      <c r="G3" s="3">
         <v>10</v>
       </c>
-      <c r="F3" s="2">
-        <v>354</v>
-      </c>
-      <c r="G3" s="2">
+      <c r="H3" s="3">
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="1">
+        <v>475</v>
+      </c>
+      <c r="D4" s="1">
         <v>570</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="1">
+      <c r="E4" s="2">
         <v>28</v>
       </c>
-      <c r="D4" s="1">
+      <c r="F4" s="2">
         <v>0.8</v>
       </c>
-      <c r="E4" s="1">
+      <c r="G4" s="3">
         <v>10</v>
       </c>
-      <c r="F4" s="2">
-        <v>354</v>
-      </c>
-      <c r="G4" s="2">
+      <c r="H4" s="3">
         <v>1500</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>245</v>
+      </c>
+      <c r="D5" s="1">
         <v>568</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="E5" s="2">
         <v>27.5</v>
       </c>
-      <c r="D5" s="1">
+      <c r="F5" s="2">
         <v>0.8</v>
       </c>
-      <c r="E5" s="1">
+      <c r="G5" s="3">
         <v>10</v>
       </c>
-      <c r="F5" s="2">
-        <v>354</v>
-      </c>
-      <c r="G5" s="2">
+      <c r="H5" s="3">
         <v>1500</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1">
+        <v>345</v>
+      </c>
+      <c r="D6" s="1">
+        <v>311</v>
+      </c>
+      <c r="E6" s="2">
         <v>40</v>
       </c>
-      <c r="D6" s="1">
+      <c r="F6" s="2">
         <v>1.7</v>
       </c>
-      <c r="E6" s="1">
+      <c r="G6" s="3">
         <v>10</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2">
+      <c r="H6" s="3">
         <v>1500</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1">
+        <v>265</v>
+      </c>
+      <c r="D7" s="1">
+        <v>425</v>
+      </c>
+      <c r="E7" s="2">
+        <v>140</v>
+      </c>
+      <c r="F7" s="3">
+        <v>3</v>
+      </c>
+      <c r="G7" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1">
+        <v>236</v>
+      </c>
+      <c r="D8" s="1">
+        <v>655</v>
+      </c>
+      <c r="E8" s="2">
+        <v>95</v>
+      </c>
+      <c r="F8" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="1">
-        <v>140</v>
-      </c>
-      <c r="D7" s="1">
+      <c r="G8" s="3">
         <v>3</v>
       </c>
-      <c r="E7" s="1">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="1">
-        <v>95</v>
-      </c>
-      <c r="D8" s="1">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="1">
+        <v>321</v>
+      </c>
+      <c r="D9" s="1">
+        <v>745</v>
+      </c>
+      <c r="E9" s="2">
+        <v>150</v>
+      </c>
+      <c r="F9" s="3">
+        <v>2</v>
+      </c>
+      <c r="G9" s="3">
         <v>5</v>
       </c>
-      <c r="E8" s="1">
-        <v>3</v>
-      </c>
-      <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1">
-        <v>150</v>
-      </c>
-      <c r="D9" s="1">
-        <v>2</v>
-      </c>
-      <c r="E9" s="1">
-        <v>5</v>
-      </c>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>

</xml_diff>